<commit_message>
chore: remove lab checkpoints and rejoin steps
Each lab folder now holds only its instruction PDF, the lab workbook
and the templates that lab uses. The checkpoints folders, the
"Checkpoint" PDF section and every rejoin instruction are removed;
labs that build on earlier work use the learner's own outputs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/labs/lab-01-excel-to-word/data/Northstar_Work_Orders.xlsx
+++ b/labs/lab-01-excel-to-word/data/Northstar_Work_Orders.xlsx
@@ -545,12 +545,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Rejoin</t>
+          <t>Use</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>This input is a deterministic checkpoint, not proof of your Copilot output.</t>
+          <t>Work on a copy saved to your OneDrive folder; keep this supplied workbook unchanged.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: simple, self-contained labs for GenAI for Engineers v2.4
Every lab now works directly on the files in its own data folder: no
extra work folder, no copying between folders and no dependence on
finishing an earlier lab. Lab 2 ships the finished Lab 1 workbook and
Word brief; Lab 6 and Lab 10 ship ready-made decks to improve.

Steps follow the C34 style: a short headline, the exact clicks, what
you should see, and one plain-English prompt (one paste, no blank
lines). Steps without a prompt get a "What you should see" checklist
box on the prompts page instead of a Copy button. Skill installs use
the OneDrive folder-upload route; SKILL.md authoring moves to an
optional Challenge.

Also: Excel desktop works on local files (no OneDrive upload), the
deck compares local upload with OneDrive references, and the v2.3
deck is superseded by v2.4.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/labs/lab-01-excel-to-word/data/Northstar_Work_Orders.xlsx
+++ b/labs/lab-01-excel-to-word/data/Northstar_Work_Orders.xlsx
@@ -550,7 +550,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Work on a copy saved to your OneDrive folder; keep this supplied workbook unchanged.</t>
+          <t>Synthetic training data. Work on this file in your lab folder.</t>
         </is>
       </c>
     </row>
@@ -7585,7 +7585,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -7642,7 +7642,7 @@
       <c r="C2" s="2" t="inlineStr">
         <is>
           <t>EXCEL - CHAT ONLY:
-Read About_This_Data and Control for Northstar Water Services. Explain what one water-pipe service work order represents, the reporting date, the five job categories and how current owners differ from proposed owners. Do not edit or infer customer impacts.</t>
+Describe this work-order table for me. How many rows are there? Are there any repeated Work_Order_IDs, or Job_Category names spelt in different ways? Don’t change anything.</t>
         </is>
       </c>
     </row>
@@ -7654,13 +7654,13 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>EXCEL - CHAT ONLY</t>
+          <t>EXCEL - ALLOW EDITING</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>EXCEL - CHAT ONLY:
-Inspect tblWorkOrders. Report row count, duplicate Work_Order_ID values, category spelling variants and missing Assigned_To. Do not edit. Treat 2026-09-30 as the fixed reporting date.</t>
+          <t>EXCEL - ALLOW EDITING:
+Copy the table to a new sheet named Raw_Export. Then remove the repeated rows, keeping one row for each Work_Order_ID, and fix the Job_Category spelling. Leave empty Assigned_To cells empty.</t>
         </is>
       </c>
     </row>
@@ -7672,15 +7672,13 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>EXCEL - PLAN</t>
+          <t>EXCEL - ALLOW EDITING</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>EXCEL - PLAN:
-Plan to retain an untouched Raw_Export copy, remove only exact duplicate records by Work_Order_ID, and standardise category spelling in tblWorkOrders. Keep dates, statuses and assignments. Ask if two records with one ID differ.
-EXCEL - ALLOW EDITING:
-Apply the reviewed plan. Keep one identical record per repeated ID. Do not guess missing owners. Reconcile the cleaned table against Control.</t>
+          <t>EXCEL - ALLOW EDITING:
+In the Checks sheet, add formulas that count the total work orders, closed, cancelled, backlog (not Closed or Cancelled), overdue backlog (due before the date in Control!B2) and unassigned backlog, and add up Cost_SGD.</t>
         </is>
       </c>
     </row>
@@ -7692,13 +7690,13 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>EXCEL - ALLOW EDITING</t>
+          <t>WORD COPILOT</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>EXCEL - ALLOW EDITING:
-In Checks calculate total rows, closed, cancelled, backlog, overdue backlog, unassigned backlog and total Cost_SGD for tblWorkOrders. Use Control!B2 as reporting date. Define backlog as Status neither Closed nor Cancelled. Add the identity total = closed + cancelled + backlog. Do not change source data.</t>
+          <t>WORD COPILOT:
+Write a one-page operations brief in this document from the uploaded Northstar_Work_Orders.xlsx. Include the reporting date, the key numbers from the Checks sheet, the backlog and overdue findings, the unassigned jobs, proposed next actions and open questions. Use only numbers from the workbook, and write UNKNOWN for anything it does not show.</t>
         </is>
       </c>
     </row>
@@ -7716,25 +7714,7 @@
       <c r="C6" s="2" t="inlineStr">
         <is>
           <t>WORD COPILOT:
-Draft a one-page Northstar operations brief from the verified evidence supplied here. Include reporting scope/date, backlog and overdue findings, current assignment issues, proposed next actions and open questions. Keep observed facts separate from proposals. Preserve numbers and definitions. Use UNKNOWN for causes, approvals or capacity decisions not evidenced.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Step 6</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>WORD COPILOT</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>WORD COPILOT:
-Audit this Northstar Water Services operations brief against the verified evidence table I supply. Return a discrepancy list for counts, cost, reporting scope, overdue definition and assignment claims. Identify missing source links as UNKNOWN. Do not change facts or approve work.</t>
+Check every number in this brief against the uploaded workbook. List any number that is different, with the correct value.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add PowerPoint design-skill lab, failure-mode Pareto and new slides
- New Lab 7: create northstar-deck-design, a PowerPoint skill that turns
  a plain deck into a branded, professional one (Segoe UI, navy header
  bar, KPI cards, footer). Ships a plain 6-slide deck and a reference
  SKILL.md. Former Labs 7-12 are renumbered 8-13; LP timetable, LG,
  deck, prompts page and lab folders follow the new sequence.
- Work orders now record a Failure_Mode. Lab 5 builds a Pareto of the
  vital few failure modes (3 of 8 = 78%); Lab 6 installs both the
  Pareto and reporting skills and adds the Pareto to the report.
- Deck: "Copilot: One Agentic AI Interface, Four Tools" hub diagram
  before Topic 1, and "Anatomy of a Skill" (on-demand trigger, name and
  description metadata, steps, reference files) before the skill labs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/labs/lab-01-excel-to-word/data/Northstar_Work_Orders.xlsx
+++ b/labs/lab-01-excel-to-word/data/Northstar_Work_Orders.xlsx
@@ -154,9 +154,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblWorkOrders" displayName="tblWorkOrders" ref="A1:M123" headerRowCount="1">
-  <autoFilter ref="A1:M123"/>
-  <tableColumns count="13">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblWorkOrders" displayName="tblWorkOrders" ref="A1:N123" headerRowCount="1">
+  <autoFilter ref="A1:N123"/>
+  <tableColumns count="14">
     <tableColumn id="1" name="Work_Order_ID"/>
     <tableColumn id="2" name="Site"/>
     <tableColumn id="3" name="Job_Category"/>
@@ -170,6 +170,7 @@
     <tableColumn id="11" name="Actual_Hours"/>
     <tableColumn id="12" name="Cost_SGD"/>
     <tableColumn id="13" name="Description"/>
+    <tableColumn id="14" name="Failure_Mode"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -565,7 +566,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M123"/>
+  <dimension ref="A1:N123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -581,6 +582,7 @@
     <col width="17" customWidth="1" min="11" max="11"/>
     <col width="17" customWidth="1" min="12" max="12"/>
     <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="17" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -649,6 +651,11 @@
           <t>Description</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Failure_Mode</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -704,6 +711,11 @@
           <t>Leak Repair scheduled or reactive task 001</t>
         </is>
       </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -757,6 +769,11 @@
       <c r="M3" s="2" t="inlineStr">
         <is>
           <t>Leak Repair scheduled or reactive task 002</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
         </is>
       </c>
     </row>
@@ -812,6 +829,11 @@
           <t>Leak Repair scheduled or reactive task 003</t>
         </is>
       </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -865,6 +887,11 @@
           <t>Leak Repair scheduled or reactive task 004</t>
         </is>
       </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -918,6 +945,11 @@
           <t>Valve Repair scheduled or reactive task 005</t>
         </is>
       </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -973,6 +1005,11 @@
           <t>Valve Repair scheduled or reactive task 006</t>
         </is>
       </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1026,6 +1063,11 @@
       <c r="M8" s="2" t="inlineStr">
         <is>
           <t>Valve Repair scheduled or reactive task 007</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
         </is>
       </c>
     </row>
@@ -1081,6 +1123,11 @@
           <t>Valve Repair scheduled or reactive task 008</t>
         </is>
       </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1134,6 +1181,11 @@
           <t>Pipe Replacement scheduled or reactive task 009</t>
         </is>
       </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1187,6 +1239,11 @@
           <t>Pipe Replacement scheduled or reactive task 010</t>
         </is>
       </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1242,6 +1299,11 @@
           <t>Pipe Replacement scheduled or reactive task 011</t>
         </is>
       </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1295,6 +1357,11 @@
       <c r="M13" s="2" t="inlineStr">
         <is>
           <t>Pipe Replacement scheduled or reactive task 012</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
         </is>
       </c>
     </row>
@@ -1346,6 +1413,11 @@
           <t>Pump Service scheduled or reactive task 013</t>
         </is>
       </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>Pump bearing wear</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1399,6 +1471,11 @@
           <t>Pump Service scheduled or reactive task 014</t>
         </is>
       </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>Pump bearing wear</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1452,6 +1529,11 @@
           <t>Pump Service scheduled or reactive task 015</t>
         </is>
       </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1507,6 +1589,11 @@
           <t>Pump Service scheduled or reactive task 016</t>
         </is>
       </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>Pressure surge</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1560,6 +1647,11 @@
       <c r="M18" s="2" t="inlineStr">
         <is>
           <t>Meter Service scheduled or reactive task 017</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
         </is>
       </c>
     </row>
@@ -1615,6 +1707,11 @@
           <t>Meter Service scheduled or reactive task 018</t>
         </is>
       </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1668,6 +1765,11 @@
           <t>Meter Service scheduled or reactive task 019</t>
         </is>
       </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1721,6 +1823,11 @@
           <t>Meter Service scheduled or reactive task 020</t>
         </is>
       </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>Meter fault</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1776,6 +1883,11 @@
           <t>Leak Repair scheduled or reactive task 021</t>
         </is>
       </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1829,6 +1941,11 @@
       <c r="M23" s="2" t="inlineStr">
         <is>
           <t>Leak Repair scheduled or reactive task 022</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
         </is>
       </c>
     </row>
@@ -1884,6 +2001,11 @@
           <t>Leak Repair scheduled or reactive task 023</t>
         </is>
       </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1937,6 +2059,11 @@
           <t>Leak Repair scheduled or reactive task 024</t>
         </is>
       </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1986,6 +2113,11 @@
           <t>Valve Repair scheduled or reactive task 025</t>
         </is>
       </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2041,6 +2173,11 @@
           <t>Valve Repair scheduled or reactive task 026</t>
         </is>
       </c>
+      <c r="N27" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2094,6 +2231,11 @@
       <c r="M28" s="2" t="inlineStr">
         <is>
           <t>Valve Repair scheduled or reactive task 027</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
         </is>
       </c>
     </row>
@@ -2149,6 +2291,11 @@
           <t>Valve Repair scheduled or reactive task 028</t>
         </is>
       </c>
+      <c r="N29" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2202,6 +2349,11 @@
           <t>Pipe Replacement scheduled or reactive task 029</t>
         </is>
       </c>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2255,6 +2407,11 @@
           <t>Pipe Replacement scheduled or reactive task 030</t>
         </is>
       </c>
+      <c r="N31" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2310,6 +2467,11 @@
           <t>Pipe Replacement scheduled or reactive task 031</t>
         </is>
       </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2363,6 +2525,11 @@
       <c r="M33" s="2" t="inlineStr">
         <is>
           <t>Pipe Replacement scheduled or reactive task 032</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
         </is>
       </c>
     </row>
@@ -2418,6 +2585,11 @@
           <t>Pump Service scheduled or reactive task 033</t>
         </is>
       </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>Pump bearing wear</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2471,6 +2643,11 @@
           <t>Pump Service scheduled or reactive task 034</t>
         </is>
       </c>
+      <c r="N35" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2524,6 +2701,11 @@
           <t>Pump Service scheduled or reactive task 035</t>
         </is>
       </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2579,6 +2761,11 @@
           <t>Pump Service scheduled or reactive task 036</t>
         </is>
       </c>
+      <c r="N37" s="2" t="inlineStr">
+        <is>
+          <t>Pump bearing wear</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2632,6 +2819,11 @@
       <c r="M38" s="2" t="inlineStr">
         <is>
           <t>Meter Service scheduled or reactive task 037</t>
+        </is>
+      </c>
+      <c r="N38" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
         </is>
       </c>
     </row>
@@ -2687,6 +2879,11 @@
           <t>Meter Service scheduled or reactive task 038</t>
         </is>
       </c>
+      <c r="N39" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2740,6 +2937,11 @@
           <t>Meter Service scheduled or reactive task 039</t>
         </is>
       </c>
+      <c r="N40" s="2" t="inlineStr">
+        <is>
+          <t>Meter fault</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2793,6 +2995,11 @@
           <t>Meter Service scheduled or reactive task 040</t>
         </is>
       </c>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2848,6 +3055,11 @@
           <t>Leak Repair scheduled or reactive task 041</t>
         </is>
       </c>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2901,6 +3113,11 @@
       <c r="M43" s="2" t="inlineStr">
         <is>
           <t>Leak Repair scheduled or reactive task 042</t>
+        </is>
+      </c>
+      <c r="N43" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
         </is>
       </c>
     </row>
@@ -2956,6 +3173,11 @@
           <t>Leak Repair scheduled or reactive task 043</t>
         </is>
       </c>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>Third-party damage</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3009,6 +3231,11 @@
           <t>Leak Repair scheduled or reactive task 044</t>
         </is>
       </c>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3062,6 +3289,11 @@
           <t>Valve Repair scheduled or reactive task 045</t>
         </is>
       </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3117,6 +3349,11 @@
           <t>Valve Repair scheduled or reactive task 046</t>
         </is>
       </c>
+      <c r="N47" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -3170,6 +3407,11 @@
       <c r="M48" s="2" t="inlineStr">
         <is>
           <t>Valve Repair scheduled or reactive task 047</t>
+        </is>
+      </c>
+      <c r="N48" s="2" t="inlineStr">
+        <is>
+          <t>Pressure surge</t>
         </is>
       </c>
     </row>
@@ -3225,6 +3467,11 @@
           <t>Valve Repair scheduled or reactive task 048</t>
         </is>
       </c>
+      <c r="N49" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3274,6 +3521,11 @@
           <t>Pipe Replacement scheduled or reactive task 049</t>
         </is>
       </c>
+      <c r="N50" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3327,6 +3579,11 @@
           <t>Pipe Replacement scheduled or reactive task 050</t>
         </is>
       </c>
+      <c r="N51" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3382,6 +3639,11 @@
           <t>Pipe Replacement scheduled or reactive task 051</t>
         </is>
       </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>Pressure surge</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3435,6 +3697,11 @@
       <c r="M53" s="2" t="inlineStr">
         <is>
           <t>Pipe Replacement scheduled or reactive task 052</t>
+        </is>
+      </c>
+      <c r="N53" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
         </is>
       </c>
     </row>
@@ -3490,6 +3757,11 @@
           <t>Pump Service scheduled or reactive task 053</t>
         </is>
       </c>
+      <c r="N54" s="2" t="inlineStr">
+        <is>
+          <t>Pump bearing wear</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3543,6 +3815,11 @@
           <t>Pump Service scheduled or reactive task 054</t>
         </is>
       </c>
+      <c r="N55" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3596,6 +3873,11 @@
           <t>Pump Service scheduled or reactive task 055</t>
         </is>
       </c>
+      <c r="N56" s="2" t="inlineStr">
+        <is>
+          <t>Pressure surge</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -3651,6 +3933,11 @@
           <t>Pump Service scheduled or reactive task 056</t>
         </is>
       </c>
+      <c r="N57" s="2" t="inlineStr">
+        <is>
+          <t>Pump bearing wear</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3704,6 +3991,11 @@
       <c r="M58" s="2" t="inlineStr">
         <is>
           <t>Meter Service scheduled or reactive task 057</t>
+        </is>
+      </c>
+      <c r="N58" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
         </is>
       </c>
     </row>
@@ -3759,6 +4051,11 @@
           <t>Meter Service scheduled or reactive task 058</t>
         </is>
       </c>
+      <c r="N59" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3812,6 +4109,11 @@
           <t>Meter Service scheduled or reactive task 059</t>
         </is>
       </c>
+      <c r="N60" s="2" t="inlineStr">
+        <is>
+          <t>Blockage</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3865,6 +4167,11 @@
           <t>Meter Service scheduled or reactive task 060</t>
         </is>
       </c>
+      <c r="N61" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3920,6 +4227,11 @@
           <t>Leak Repair scheduled or reactive task 061</t>
         </is>
       </c>
+      <c r="N62" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -3973,6 +4285,11 @@
       <c r="M63" s="2" t="inlineStr">
         <is>
           <t>Leak Repair scheduled or reactive task 062</t>
+        </is>
+      </c>
+      <c r="N63" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
         </is>
       </c>
     </row>
@@ -4028,6 +4345,11 @@
           <t>Leak Repair scheduled or reactive task 063</t>
         </is>
       </c>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -4081,6 +4403,11 @@
           <t>Leak Repair scheduled or reactive task 064</t>
         </is>
       </c>
+      <c r="N65" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4134,6 +4461,11 @@
           <t>Valve Repair scheduled or reactive task 065</t>
         </is>
       </c>
+      <c r="N66" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -4189,6 +4521,11 @@
           <t>Valve Repair scheduled or reactive task 066</t>
         </is>
       </c>
+      <c r="N67" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -4242,6 +4579,11 @@
       <c r="M68" s="2" t="inlineStr">
         <is>
           <t>Valve Repair scheduled or reactive task 067</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
         </is>
       </c>
     </row>
@@ -4297,6 +4639,11 @@
           <t>Valve Repair scheduled or reactive task 068</t>
         </is>
       </c>
+      <c r="N69" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -4350,6 +4697,11 @@
           <t>Pipe Replacement scheduled or reactive task 069</t>
         </is>
       </c>
+      <c r="N70" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4403,6 +4755,11 @@
           <t>Pipe Replacement scheduled or reactive task 070</t>
         </is>
       </c>
+      <c r="N71" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4458,6 +4815,11 @@
           <t>Pipe Replacement scheduled or reactive task 071</t>
         </is>
       </c>
+      <c r="N72" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4511,6 +4873,11 @@
       <c r="M73" s="2" t="inlineStr">
         <is>
           <t>Pipe Replacement scheduled or reactive task 072</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
         </is>
       </c>
     </row>
@@ -4562,6 +4929,11 @@
           <t>Pump Service scheduled or reactive task 073</t>
         </is>
       </c>
+      <c r="N74" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4615,6 +4987,11 @@
           <t>Pump Service scheduled or reactive task 074</t>
         </is>
       </c>
+      <c r="N75" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4668,6 +5045,11 @@
           <t>Pump Service scheduled or reactive task 075</t>
         </is>
       </c>
+      <c r="N76" s="2" t="inlineStr">
+        <is>
+          <t>Pump bearing wear</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -4723,6 +5105,11 @@
           <t>Pump Service scheduled or reactive task 076</t>
         </is>
       </c>
+      <c r="N77" s="2" t="inlineStr">
+        <is>
+          <t>Pump bearing wear</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -4776,6 +5163,11 @@
       <c r="M78" s="2" t="inlineStr">
         <is>
           <t>Meter Service scheduled or reactive task 077</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
         </is>
       </c>
     </row>
@@ -4831,6 +5223,11 @@
           <t>Meter Service scheduled or reactive task 078</t>
         </is>
       </c>
+      <c r="N79" s="2" t="inlineStr">
+        <is>
+          <t>Meter fault</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -4884,6 +5281,11 @@
           <t>Meter Service scheduled or reactive task 079</t>
         </is>
       </c>
+      <c r="N80" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -4937,6 +5339,11 @@
           <t>Meter Service scheduled or reactive task 080</t>
         </is>
       </c>
+      <c r="N81" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -4992,6 +5399,11 @@
           <t>Leak Repair scheduled or reactive task 081</t>
         </is>
       </c>
+      <c r="N82" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -5045,6 +5457,11 @@
       <c r="M83" s="2" t="inlineStr">
         <is>
           <t>Leak Repair scheduled or reactive task 082</t>
+        </is>
+      </c>
+      <c r="N83" s="2" t="inlineStr">
+        <is>
+          <t>Third-party damage</t>
         </is>
       </c>
     </row>
@@ -5100,6 +5517,11 @@
           <t>Leak Repair scheduled or reactive task 083</t>
         </is>
       </c>
+      <c r="N84" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -5153,6 +5575,11 @@
           <t>Leak Repair scheduled or reactive task 084</t>
         </is>
       </c>
+      <c r="N85" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -5202,6 +5629,11 @@
           <t>Valve Repair scheduled or reactive task 085</t>
         </is>
       </c>
+      <c r="N86" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -5257,6 +5689,11 @@
           <t>Valve Repair scheduled or reactive task 086</t>
         </is>
       </c>
+      <c r="N87" s="2" t="inlineStr">
+        <is>
+          <t>Pressure surge</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -5310,6 +5747,11 @@
       <c r="M88" s="2" t="inlineStr">
         <is>
           <t>Valve Repair scheduled or reactive task 087</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
         </is>
       </c>
     </row>
@@ -5365,6 +5807,11 @@
           <t>Valve Repair scheduled or reactive task 088</t>
         </is>
       </c>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -5418,6 +5865,11 @@
           <t>Pipe Replacement scheduled or reactive task 089</t>
         </is>
       </c>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -5471,6 +5923,11 @@
           <t>Pipe Replacement scheduled or reactive task 090</t>
         </is>
       </c>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
+          <t>Pressure surge</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -5526,6 +5983,11 @@
           <t>Pipe Replacement scheduled or reactive task 091</t>
         </is>
       </c>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -5579,6 +6041,11 @@
       <c r="M93" s="2" t="inlineStr">
         <is>
           <t>Pipe Replacement scheduled or reactive task 092</t>
+        </is>
+      </c>
+      <c r="N93" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
         </is>
       </c>
     </row>
@@ -5634,6 +6101,11 @@
           <t>Pump Service scheduled or reactive task 093</t>
         </is>
       </c>
+      <c r="N94" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -5687,6 +6159,11 @@
           <t>Pump Service scheduled or reactive task 094</t>
         </is>
       </c>
+      <c r="N95" s="2" t="inlineStr">
+        <is>
+          <t>Pressure surge</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -5740,6 +6217,11 @@
           <t>Pump Service scheduled or reactive task 095</t>
         </is>
       </c>
+      <c r="N96" s="2" t="inlineStr">
+        <is>
+          <t>Pump bearing wear</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -5795,6 +6277,11 @@
           <t>Pump Service scheduled or reactive task 096</t>
         </is>
       </c>
+      <c r="N97" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -5848,6 +6335,11 @@
       <c r="M98" s="2" t="inlineStr">
         <is>
           <t>Meter Service scheduled or reactive task 097</t>
+        </is>
+      </c>
+      <c r="N98" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
         </is>
       </c>
     </row>
@@ -5903,6 +6395,11 @@
           <t>Meter Service scheduled or reactive task 098</t>
         </is>
       </c>
+      <c r="N99" s="2" t="inlineStr">
+        <is>
+          <t>Blockage</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -5956,6 +6453,11 @@
           <t>Meter Service scheduled or reactive task 099</t>
         </is>
       </c>
+      <c r="N100" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -6009,6 +6511,11 @@
           <t>Meter Service scheduled or reactive task 100</t>
         </is>
       </c>
+      <c r="N101" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -6064,6 +6571,11 @@
           <t>Leak Repair scheduled or reactive task 101</t>
         </is>
       </c>
+      <c r="N102" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -6117,6 +6629,11 @@
       <c r="M103" s="2" t="inlineStr">
         <is>
           <t>Leak Repair scheduled or reactive task 102</t>
+        </is>
+      </c>
+      <c r="N103" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
         </is>
       </c>
     </row>
@@ -6172,6 +6689,11 @@
           <t>Leak Repair scheduled or reactive task 103</t>
         </is>
       </c>
+      <c r="N104" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -6225,6 +6747,11 @@
           <t>Leak Repair scheduled or reactive task 104</t>
         </is>
       </c>
+      <c r="N105" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -6278,6 +6805,11 @@
           <t>Valve Repair scheduled or reactive task 105</t>
         </is>
       </c>
+      <c r="N106" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -6333,6 +6865,11 @@
           <t>Valve Repair scheduled or reactive task 106</t>
         </is>
       </c>
+      <c r="N107" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -6386,6 +6923,11 @@
       <c r="M108" s="2" t="inlineStr">
         <is>
           <t>Valve Repair scheduled or reactive task 107</t>
+        </is>
+      </c>
+      <c r="N108" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
         </is>
       </c>
     </row>
@@ -6441,6 +6983,11 @@
           <t>Valve Repair scheduled or reactive task 108</t>
         </is>
       </c>
+      <c r="N109" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -6490,6 +7037,11 @@
           <t>Pipe Replacement scheduled or reactive task 109</t>
         </is>
       </c>
+      <c r="N110" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -6543,6 +7095,11 @@
           <t>Pipe Replacement scheduled or reactive task 110</t>
         </is>
       </c>
+      <c r="N111" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -6598,6 +7155,11 @@
           <t>Pipe Replacement scheduled or reactive task 111</t>
         </is>
       </c>
+      <c r="N112" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -6651,6 +7213,11 @@
       <c r="M113" s="2" t="inlineStr">
         <is>
           <t>Pipe Replacement scheduled or reactive task 112</t>
+        </is>
+      </c>
+      <c r="N113" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
         </is>
       </c>
     </row>
@@ -6706,6 +7273,11 @@
           <t>Pump Service scheduled or reactive task 113</t>
         </is>
       </c>
+      <c r="N114" s="2" t="inlineStr">
+        <is>
+          <t>Pressure surge</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -6759,6 +7331,11 @@
           <t>Pump Service scheduled or reactive task 114</t>
         </is>
       </c>
+      <c r="N115" s="2" t="inlineStr">
+        <is>
+          <t>Pump bearing wear</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -6812,6 +7389,11 @@
           <t>Pump Service scheduled or reactive task 115</t>
         </is>
       </c>
+      <c r="N116" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -6867,6 +7449,11 @@
           <t>Pump Service scheduled or reactive task 116</t>
         </is>
       </c>
+      <c r="N117" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -6920,6 +7507,11 @@
       <c r="M118" s="2" t="inlineStr">
         <is>
           <t>Meter Service scheduled or reactive task 117</t>
+        </is>
+      </c>
+      <c r="N118" s="2" t="inlineStr">
+        <is>
+          <t>Meter fault</t>
         </is>
       </c>
     </row>
@@ -6975,6 +7567,11 @@
           <t>Meter Service scheduled or reactive task 118</t>
         </is>
       </c>
+      <c r="N119" s="2" t="inlineStr">
+        <is>
+          <t>Corrosion</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -7028,6 +7625,11 @@
           <t>Meter Service scheduled or reactive task 119</t>
         </is>
       </c>
+      <c r="N120" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -7081,6 +7683,11 @@
           <t>Meter Service scheduled or reactive task 120</t>
         </is>
       </c>
+      <c r="N121" s="2" t="inlineStr">
+        <is>
+          <t>Joint seal leak</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -7134,6 +7741,11 @@
           <t>Valve Repair scheduled or reactive task 005</t>
         </is>
       </c>
+      <c r="N122" s="2" t="inlineStr">
+        <is>
+          <t>Valve seat wear</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -7185,6 +7797,11 @@
       <c r="M123" s="2" t="inlineStr">
         <is>
           <t>Meter Service scheduled or reactive task 020</t>
+        </is>
+      </c>
+      <c r="N123" s="2" t="inlineStr">
+        <is>
+          <t>Meter fault</t>
         </is>
       </c>
     </row>

</xml_diff>